<commit_message>
NAKO-5 NAKO files for P2 initial harmonisation
</commit_message>
<xml_diff>
--- a/analyst/Ines/rmonize/data_proc_elem/DPE_NAKO_INES.xlsx
+++ b/analyst/Ines/rmonize/data_proc_elem/DPE_NAKO_INES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\use-cases-harmonisation\analyst\Ines\rmonize\data_proc_elem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\analyst\Ines\rmonize\data_proc_elem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB98EF93-84A2-46EF-936A-5615FE41ABEF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D6ACFF6-35CD-4AFB-8799-CF8622242508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-525" yWindow="1200" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -339,9 +339,6 @@
     <t>a_nu_mna</t>
   </si>
   <si>
-    <t>a_nu_mna; a_nu_mk</t>
-  </si>
-  <si>
     <t>a_nu_mna/a_nu_mk</t>
   </si>
   <si>
@@ -406,6 +403,9 @@
   </si>
   <si>
     <t>anthro_taillenumfang_fup</t>
+  </si>
+  <si>
+    <t>a_nu_mna;a_nu_mk</t>
   </si>
 </sst>
 </file>
@@ -474,7 +474,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -490,9 +490,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -530,9 +530,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -565,26 +565,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -617,26 +600,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -814,7 +780,7 @@
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
   <dimension ref="A1:K36"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="67.5703125" bestFit="1" customWidth="1"/>
@@ -1006,7 +972,7 @@
         <v>82</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J6" s="4" t="s">
         <v>83</v>
@@ -1038,7 +1004,7 @@
         <v>82</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J7" s="4" t="s">
         <v>83</v>
@@ -1117,7 +1083,7 @@
         <v>80</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>82</v>
@@ -1126,7 +1092,7 @@
         <v>82</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J10" s="4" t="s">
         <v>83</v>
@@ -1149,7 +1115,7 @@
         <v>80</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>82</v>
@@ -1158,7 +1124,7 @@
         <v>82</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J11" s="4" t="s">
         <v>83</v>
@@ -1190,7 +1156,7 @@
         <v>82</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J12" s="4" t="s">
         <v>83</v>
@@ -1222,7 +1188,7 @@
         <v>82</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J13" s="4" t="s">
         <v>83</v>
@@ -1328,7 +1294,7 @@
         <v>80</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>82</v>
@@ -1337,7 +1303,7 @@
         <v>82</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J17" s="4" t="s">
         <v>83</v>
@@ -1360,7 +1326,7 @@
         <v>80</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>82</v>
@@ -1389,7 +1355,7 @@
         <v>80</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G19" s="4" t="s">
         <v>82</v>
@@ -1425,7 +1391,7 @@
         <v>93</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="4" t="s">
@@ -1455,7 +1421,7 @@
         <v>93</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="4" t="s">
@@ -1485,7 +1451,7 @@
         <v>93</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I22" s="2"/>
       <c r="J22" s="4" t="s">
@@ -1515,7 +1481,7 @@
         <v>93</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I23" s="2"/>
       <c r="J23" s="4" t="s">
@@ -1545,7 +1511,7 @@
         <v>93</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I24" s="2"/>
       <c r="J24" s="4" t="s">
@@ -1597,13 +1563,13 @@
         <v>80</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G26" s="4" t="s">
         <v>93</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="4" t="s">
@@ -1627,13 +1593,13 @@
         <v>80</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G27" s="4" t="s">
         <v>93</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I27" s="2"/>
       <c r="J27" s="4" t="s">
@@ -1657,13 +1623,13 @@
         <v>80</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G28" s="4" t="s">
         <v>93</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I28" s="2"/>
       <c r="J28" s="4" t="s">
@@ -1743,13 +1709,13 @@
         <v>80</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G31" s="4" t="s">
         <v>93</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="4" t="s">
@@ -1773,13 +1739,13 @@
         <v>80</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G32" s="4" t="s">
         <v>93</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I32" s="2"/>
       <c r="J32" s="4" t="s">
@@ -1889,13 +1855,13 @@
         <v>80</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>93</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2" t="s">

</xml_diff>